<commit_message>
Update 6O_mapping.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/6O_mapping.xlsx
+++ b/6O_mapping.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
   <si>
     <t>BUILD</t>
   </si>
@@ -133,12 +133,6 @@
   </si>
   <si>
     <t>Chiller sustained out-of-range: ext_valve_flow_out_of_rack=0.0 (limit [2.5, 1000.0]) failed 3/3 times; overall_delta_pressure_psi=-0.1 (limit [17.0, 25.0]) failed 3/3 times</t>
-  </si>
-  <si>
-    <t>cpo_collect_linkup-[meas,ei,li,oil,oli,fc,opm,eip,eocl,tp,prp,prb,prbl],[prbl:nan,2,6,4,8,15,139.75,12.76,8.69,6.32,-22.08,nan,nan],[prb:nan,2,6,4,8,15,139.75,12.76,8.69,6.32,-22.08,nan,nan],[prp:-22.08,2,6,4,8,15,139.75,12.76,8.69,6.32,-22.08,nan,nan],[prbl:nan,2,6,4,9,15,139.75,12.82,8.63,6.32,-21.87,nan,nan],[prb:nan,2,6,4,9,15,139.75,12.82,8.63,6.32,-21.87,nan,nan],[prp:-21.87,2,6,4,9,15,139.75,12.82,8.63,6.32,-21.87,nan,nan],[prbl:nan,2,6,4,10,15,139.75,12.86,8.59,6.46,-22.08,nan,nan],[prb:nan,2,6,4,10,15,139.75,12.86,8.59,6.46,-22.08,nan,nan],[prp:-22.08,2,6,4,10,15,139.75,12.86,8.59,6.46,-22.08,nan,nan],[prbl:nan,2,6,4,11,15,139.75,12.73,8.72,6.32,-22.37,nan,nan],[prb:nan,2,6,4,11,15,139.75,12.73,8.72,6.32,-22.37,nan,nan],[prp:-22.37,2,6,4,11,15,139.75,12.73,8.72,6.32,-22.37,nan,nan]</t>
-  </si>
-  <si>
-    <t>OE12 lane 5 mmc46 bad rx</t>
   </si>
   <si>
     <t>FULL SYS</t>
@@ -494,12 +488,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="5" max="5" width="8.25" customWidth="1"/>
-    <col min="10" max="10" width="25.75" customWidth="1"/>
+    <col min="3" max="3" width="17.375" customWidth="1"/>
+    <col min="4" max="4" width="10.375" customWidth="1"/>
+    <col min="5" max="5" width="15.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">
@@ -522,7 +516,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -581,7 +575,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -622,7 +616,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -654,7 +648,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -689,7 +683,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -717,20 +711,6 @@
       </c>
       <c r="N5" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="L6" t="s">
-        <v>6</v>
-      </c>
-      <c r="M6" t="s">
-        <v>32</v>
-      </c>
-      <c r="N6" t="s">
-        <v>37</v>
-      </c>
-      <c r="O6" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>